<commit_message>
Batch size 8 and low temps for wd 0.003
</commit_message>
<xml_diff>
--- a/data/Comparing_Dynamics (1).xlsx
+++ b/data/Comparing_Dynamics (1).xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1070" uniqueCount="254">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1152" uniqueCount="276">
   <si>
     <t>Datset</t>
   </si>
@@ -737,6 +737,72 @@
     <t>noble-morning-428</t>
   </si>
   <si>
+    <t>noble-forest-468</t>
+  </si>
+  <si>
+    <t>curious-bee-465</t>
+  </si>
+  <si>
+    <t>driven-violet-463</t>
+  </si>
+  <si>
+    <t>peach-valley-457</t>
+  </si>
+  <si>
+    <t>azure-energy-448</t>
+  </si>
+  <si>
+    <t>smart-glitter-470</t>
+  </si>
+  <si>
+    <t>misty-snowball-469</t>
+  </si>
+  <si>
+    <t>winter-cloud-467</t>
+  </si>
+  <si>
+    <t>avid-star-466</t>
+  </si>
+  <si>
+    <t>easy-hill-464</t>
+  </si>
+  <si>
+    <t>vocal-wood-462</t>
+  </si>
+  <si>
+    <t>noble-firebrand-461</t>
+  </si>
+  <si>
+    <t>desert-sky-460</t>
+  </si>
+  <si>
+    <t>misty-energy-459</t>
+  </si>
+  <si>
+    <t>stilted-cloud-458</t>
+  </si>
+  <si>
+    <t>jolly-galaxy-456</t>
+  </si>
+  <si>
+    <t>hearty-plasma-455</t>
+  </si>
+  <si>
+    <t>exalted-oath-454</t>
+  </si>
+  <si>
+    <t>peach-breeze-453</t>
+  </si>
+  <si>
+    <t>pious-hill-451</t>
+  </si>
+  <si>
+    <t>equilibrate_sgd_weight_decay.ipynb</t>
+  </si>
+  <si>
+    <t>Equilibrate with the fluctuation-dissipation relation bit. + weight decay that actually converges!</t>
+  </si>
+  <si>
     <t>equilibrate_sgd_checkpoints.ipynb</t>
   </si>
   <si>
@@ -1335,7 +1401,7 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" headerRowCount="0" ref="A2:F111" displayName="Table_1" name="Table_1" id="2">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" headerRowCount="0" ref="A2:F131" displayName="Table_1" name="Table_1" id="2">
   <tableColumns count="6">
     <tableColumn name="Column1" id="1"/>
     <tableColumn name="Column2" id="2"/>
@@ -12777,6 +12843,406 @@
         <v>18</v>
       </c>
     </row>
+    <row r="112">
+      <c r="A112" s="43" t="s">
+        <v>240</v>
+      </c>
+      <c r="B112" s="57">
+        <v>8.0</v>
+      </c>
+      <c r="C112" s="43" t="s">
+        <v>18</v>
+      </c>
+      <c r="D112" s="43" t="s">
+        <v>43</v>
+      </c>
+      <c r="E112" s="57">
+        <v>49.0</v>
+      </c>
+      <c r="F112" s="43" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" s="43" t="s">
+        <v>241</v>
+      </c>
+      <c r="B113" s="57">
+        <v>8.0</v>
+      </c>
+      <c r="C113" s="43" t="s">
+        <v>18</v>
+      </c>
+      <c r="D113" s="43" t="s">
+        <v>43</v>
+      </c>
+      <c r="E113" s="57">
+        <v>39.0</v>
+      </c>
+      <c r="F113" s="43" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" s="43" t="s">
+        <v>242</v>
+      </c>
+      <c r="B114" s="57">
+        <v>8.0</v>
+      </c>
+      <c r="C114" s="43" t="s">
+        <v>18</v>
+      </c>
+      <c r="D114" s="43" t="s">
+        <v>43</v>
+      </c>
+      <c r="E114" s="57">
+        <v>29.0</v>
+      </c>
+      <c r="F114" s="43" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" s="43" t="s">
+        <v>243</v>
+      </c>
+      <c r="B115" s="57">
+        <v>8.0</v>
+      </c>
+      <c r="C115" s="43" t="s">
+        <v>18</v>
+      </c>
+      <c r="D115" s="43" t="s">
+        <v>43</v>
+      </c>
+      <c r="E115" s="57">
+        <v>19.0</v>
+      </c>
+      <c r="F115" s="43" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" s="43" t="s">
+        <v>244</v>
+      </c>
+      <c r="B116" s="57">
+        <v>8.0</v>
+      </c>
+      <c r="C116" s="43" t="s">
+        <v>18</v>
+      </c>
+      <c r="D116" s="43" t="s">
+        <v>43</v>
+      </c>
+      <c r="E116" s="57">
+        <v>11.0</v>
+      </c>
+      <c r="F116" s="43" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" s="43" t="s">
+        <v>245</v>
+      </c>
+      <c r="B117" s="57">
+        <v>1024.0</v>
+      </c>
+      <c r="C117" s="43" t="s">
+        <v>18</v>
+      </c>
+      <c r="D117" s="43" t="s">
+        <v>43</v>
+      </c>
+      <c r="E117" s="57">
+        <v>49.0</v>
+      </c>
+      <c r="F117" s="43" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" s="43" t="s">
+        <v>246</v>
+      </c>
+      <c r="B118" s="57">
+        <v>1024.0</v>
+      </c>
+      <c r="C118" s="43" t="s">
+        <v>18</v>
+      </c>
+      <c r="D118" s="43" t="s">
+        <v>43</v>
+      </c>
+      <c r="E118" s="57">
+        <v>39.0</v>
+      </c>
+      <c r="F118" s="43" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" s="43" t="s">
+        <v>247</v>
+      </c>
+      <c r="B119" s="57">
+        <v>1024.0</v>
+      </c>
+      <c r="C119" s="43" t="s">
+        <v>18</v>
+      </c>
+      <c r="D119" s="43" t="s">
+        <v>43</v>
+      </c>
+      <c r="E119" s="57">
+        <v>29.0</v>
+      </c>
+      <c r="F119" s="43" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" s="43" t="s">
+        <v>248</v>
+      </c>
+      <c r="B120" s="57">
+        <v>1024.0</v>
+      </c>
+      <c r="C120" s="43" t="s">
+        <v>18</v>
+      </c>
+      <c r="D120" s="43" t="s">
+        <v>43</v>
+      </c>
+      <c r="E120" s="57">
+        <v>19.0</v>
+      </c>
+      <c r="F120" s="43" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" s="43" t="s">
+        <v>249</v>
+      </c>
+      <c r="B121" s="57">
+        <v>1024.0</v>
+      </c>
+      <c r="C121" s="43" t="s">
+        <v>18</v>
+      </c>
+      <c r="D121" s="43" t="s">
+        <v>43</v>
+      </c>
+      <c r="E121" s="57">
+        <v>11.0</v>
+      </c>
+      <c r="F121" s="43" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" s="43" t="s">
+        <v>250</v>
+      </c>
+      <c r="B122" s="57">
+        <v>256.0</v>
+      </c>
+      <c r="C122" s="43" t="s">
+        <v>18</v>
+      </c>
+      <c r="D122" s="43" t="s">
+        <v>43</v>
+      </c>
+      <c r="E122" s="57">
+        <v>49.0</v>
+      </c>
+      <c r="F122" s="43" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" s="43" t="s">
+        <v>251</v>
+      </c>
+      <c r="B123" s="57">
+        <v>256.0</v>
+      </c>
+      <c r="C123" s="43" t="s">
+        <v>18</v>
+      </c>
+      <c r="D123" s="43" t="s">
+        <v>43</v>
+      </c>
+      <c r="E123" s="57">
+        <v>39.0</v>
+      </c>
+      <c r="F123" s="43" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" s="43" t="s">
+        <v>252</v>
+      </c>
+      <c r="B124" s="57">
+        <v>256.0</v>
+      </c>
+      <c r="C124" s="43" t="s">
+        <v>18</v>
+      </c>
+      <c r="D124" s="43" t="s">
+        <v>43</v>
+      </c>
+      <c r="E124" s="57">
+        <v>29.0</v>
+      </c>
+      <c r="F124" s="43" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" s="43" t="s">
+        <v>253</v>
+      </c>
+      <c r="B125" s="57">
+        <v>256.0</v>
+      </c>
+      <c r="C125" s="43" t="s">
+        <v>18</v>
+      </c>
+      <c r="D125" s="43" t="s">
+        <v>43</v>
+      </c>
+      <c r="E125" s="57">
+        <v>19.0</v>
+      </c>
+      <c r="F125" s="43" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" s="43" t="s">
+        <v>254</v>
+      </c>
+      <c r="B126" s="57">
+        <v>256.0</v>
+      </c>
+      <c r="C126" s="43" t="s">
+        <v>18</v>
+      </c>
+      <c r="D126" s="43" t="s">
+        <v>43</v>
+      </c>
+      <c r="E126" s="57">
+        <v>11.0</v>
+      </c>
+      <c r="F126" s="43" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" s="43" t="s">
+        <v>255</v>
+      </c>
+      <c r="B127" s="57">
+        <v>128.0</v>
+      </c>
+      <c r="C127" s="43" t="s">
+        <v>18</v>
+      </c>
+      <c r="D127" s="43" t="s">
+        <v>43</v>
+      </c>
+      <c r="E127" s="57">
+        <v>49.0</v>
+      </c>
+      <c r="F127" s="43" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" s="43" t="s">
+        <v>256</v>
+      </c>
+      <c r="B128" s="57">
+        <v>128.0</v>
+      </c>
+      <c r="C128" s="43" t="s">
+        <v>18</v>
+      </c>
+      <c r="D128" s="43" t="s">
+        <v>43</v>
+      </c>
+      <c r="E128" s="57">
+        <v>39.0</v>
+      </c>
+      <c r="F128" s="43" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" s="43" t="s">
+        <v>257</v>
+      </c>
+      <c r="B129" s="57">
+        <v>128.0</v>
+      </c>
+      <c r="C129" s="43" t="s">
+        <v>18</v>
+      </c>
+      <c r="D129" s="43" t="s">
+        <v>43</v>
+      </c>
+      <c r="E129" s="57">
+        <v>29.0</v>
+      </c>
+      <c r="F129" s="43" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" s="43" t="s">
+        <v>258</v>
+      </c>
+      <c r="B130" s="57">
+        <v>128.0</v>
+      </c>
+      <c r="C130" s="43" t="s">
+        <v>18</v>
+      </c>
+      <c r="D130" s="43" t="s">
+        <v>43</v>
+      </c>
+      <c r="E130" s="57">
+        <v>19.0</v>
+      </c>
+      <c r="F130" s="43" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" s="43" t="s">
+        <v>259</v>
+      </c>
+      <c r="B131" s="57">
+        <v>128.0</v>
+      </c>
+      <c r="C131" s="43" t="s">
+        <v>18</v>
+      </c>
+      <c r="D131" s="43" t="s">
+        <v>43</v>
+      </c>
+      <c r="E131" s="57">
+        <v>11.0</v>
+      </c>
+      <c r="F131" s="43" t="s">
+        <v>71</v>
+      </c>
+    </row>
   </sheetData>
   <drawing r:id="rId1"/>
   <tableParts count="1">
@@ -12795,37 +13261,46 @@
     <col customWidth="1" min="1" max="1" width="29.88"/>
   </cols>
   <sheetData>
+    <row r="3">
+      <c r="A3" s="59" t="s">
+        <v>260</v>
+      </c>
+      <c r="B3" s="44" t="s">
+        <v>261</v>
+      </c>
+    </row>
     <row r="4">
       <c r="A4" s="59" t="s">
-        <v>240</v>
+        <v>262</v>
       </c>
       <c r="B4" s="44" t="s">
-        <v>241</v>
+        <v>263</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="59" t="s">
-        <v>242</v>
+        <v>264</v>
       </c>
       <c r="B5" s="44" t="s">
-        <v>243</v>
+        <v>265</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="60" t="s">
-        <v>244</v>
+        <v>266</v>
       </c>
       <c r="B6" s="44" t="s">
-        <v>245</v>
+        <v>267</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink r:id="rId1" location="scrollTo=bHQrT25j2mZH" ref="A4"/>
-    <hyperlink r:id="rId2" location="scrollTo=fe94d4fc" ref="A5"/>
-    <hyperlink r:id="rId3" location="scrollTo=zrBZV4x86Q3H" ref="A6"/>
+    <hyperlink r:id="rId1" location="scrollTo=29mgvzAuMjkK" ref="A3"/>
+    <hyperlink r:id="rId2" location="scrollTo=bHQrT25j2mZH" ref="A4"/>
+    <hyperlink r:id="rId3" location="scrollTo=fe94d4fc" ref="A5"/>
+    <hyperlink r:id="rId4" location="scrollTo=zrBZV4x86Q3H" ref="A6"/>
   </hyperlinks>
-  <drawing r:id="rId4"/>
+  <drawing r:id="rId5"/>
 </worksheet>
 </file>
 
@@ -12898,10 +13373,10 @@
     </row>
     <row r="3">
       <c r="A3" s="62" t="s">
-        <v>246</v>
+        <v>268</v>
       </c>
       <c r="B3" s="62" t="s">
-        <v>247</v>
+        <v>269</v>
       </c>
       <c r="C3" s="61"/>
       <c r="D3" s="61"/>
@@ -12930,10 +13405,10 @@
     </row>
     <row r="4">
       <c r="A4" s="63" t="s">
-        <v>248</v>
+        <v>270</v>
       </c>
       <c r="B4" s="64" t="s">
-        <v>249</v>
+        <v>271</v>
       </c>
       <c r="C4" s="61"/>
       <c r="D4" s="61"/>
@@ -12962,10 +13437,10 @@
     </row>
     <row r="5">
       <c r="A5" s="64" t="s">
-        <v>250</v>
+        <v>272</v>
       </c>
       <c r="B5" s="64" t="s">
-        <v>251</v>
+        <v>273</v>
       </c>
       <c r="C5" s="61"/>
       <c r="D5" s="61"/>
@@ -12994,10 +13469,10 @@
     </row>
     <row r="6">
       <c r="A6" s="64" t="s">
-        <v>252</v>
+        <v>274</v>
       </c>
       <c r="B6" s="63" t="s">
-        <v>253</v>
+        <v>275</v>
       </c>
       <c r="C6" s="61"/>
       <c r="D6" s="61"/>

</xml_diff>